<commit_message>
feat: implement SUC standard bulk import scanner with Excel parsing and schema support
</commit_message>
<xml_diff>
--- a/context/suctemplate.xlsx
+++ b/context/suctemplate.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Quality-Assurance-System\context\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6B76F5E-8691-4EDD-B603-0F81BD697105}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2E6142F-F635-4DFF-ADA7-B6B4661F2E3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="10965" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="199">
   <si>
     <t>KRA</t>
   </si>
@@ -538,6 +538,239 @@
   </si>
   <si>
     <t>Local institutional recognition/accreditation/assessment: Institutional Sustainability Assessment (ISA)</t>
+  </si>
+  <si>
+    <t>Possible Evidences</t>
+  </si>
+  <si>
+    <t>- Accomplished template 
+- Scanned reports
+- Photos
+- Manual of Institutionalized Guidelines of the IRR of RA 10931 
+- Board resolution
+- Issued policy</t>
+  </si>
+  <si>
+    <t>- Enrollment data disaggregated by type
+- Certified list of disadvantaged students
+- Calculation sheet of percentage
+- Reports to CHEDRO
+- MOA/certificates for grants
+- Board resolutions on student inclusion</t>
+  </si>
+  <si>
+    <t>- MOA/certificate of scholarship grant
+- Enrolment data as per CHEDRO/CMO 40 s. 2008</t>
+  </si>
+  <si>
+    <t>- Accomplished template 1.4
+- Board resolution
+- Continuity plan
+- CHEDRO acknowledgement</t>
+  </si>
+  <si>
+    <t>- -Accomplished template 
+- Photo/video documentation
+- Disability Inclusion Strategy document
+- Board resolution
+- Client satisfaction survey</t>
+  </si>
+  <si>
+    <t>-Accomplished template - Enrolment data received by CHEDRO</t>
+  </si>
+  <si>
+    <t>- Template
+- COPC certificates
+- Certification of programs with pending COPC</t>
+  </si>
+  <si>
+    <t>- Template
+- Accrediting body letter
+- Certificates</t>
+  </si>
+  <si>
+    <t>- Complete faculty list certified by HR</t>
+  </si>
+  <si>
+    <t>- Template
+- Organizational structure
+- Policy/strategy
+- Photos
+- Portal/social media URL</t>
+  </si>
+  <si>
+    <t>- Template
+- Graduate data
+- CHEDRO reports</t>
+  </si>
+  <si>
+    <t>- Template
+- Certificates</t>
+  </si>
+  <si>
+    <t>- Template
+- Graduate tracer study design
+- Methodologies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-Accomplished templates 
+-Scanned copy of International Office Structure, Policies, Strategies and Programs
+-List of officers and staff
+-Copy of certificate of valid membership
+-Link to the website of the organization or network
+-Documentation of the implemented enhanced/developed program
+⎯MOA/MOU
+⎯Copy of board approval for the implementation of the enhanced program or newly-developed program
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-Accomplished template 
+-Scanned copy of the board-approved manual 
+-List of research collaborations with active MOA or MOU as evidenced by research output, etc.
+-Scanned copy of MOA/MOU, evidence of research output if applicable 
+-Scanned copy of notarized MOA or MOU 
+-Copy of budget utilization report per project received by CHED (List of completed and ongoing research projects using these laboratories).
+-Photo/Video documentation of the laboratories.
+-Proof of activities, approved research projects (MOA/MOU, notice to proceed)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-Accomplished template 
+-Scanned copy of patent certificate or journal where the article is published
+-List of PSIPOP every year 
+-Scanned copy of the ff: letter of acceptance, Proceedings, journal
+-Photo documentation 
+-Scanned copy of Award, Plaque, Certificate and other proof of award issued
+-Scanned copy of the invitation/call to participate in the competition
+-Background information of the award- giving bodies
+</t>
+  </si>
+  <si>
+    <t>-Accomplished template 
+-Total number of researches with registered intellectual property
+-Scanned copy of Certificates
+-Proof that the output was utilized for commercial and industrial purposes 
+-Scanned copy of Certificates 
+-Exported list of journals from the website
+-Direct link to the research output if published
+-Scanned copy of the following:
+-first page of journal articles; abstract
+-cover and publication pages (with approval date and/or edition notice) 
+-Print screen from Google Scholar/Internet indicating the title of papers citing the paper
+-Video documentation
+-Review from other artists or authorities in the field 
+-Scanned copy of MOA/MOU -Scanned copy of certificate/plaque
+-Profile of the professor given the award.
+-proof of sponsorship, if applicable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-Accomplished template 
+-Scanned copy of the board-approved Extension Policy; resolution for those without board-approval
+-Organizational structure
+-appointment of the designated officer and full-time staff
+-photo document of the office
+-Copy of Governing board-approved PRE or WFP or its equivalent (GAA + GIA or IGI)
+-Copy of Proponents brief with line item budget (LIB) showing SUC and partner share
+-Audited financial report
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-Accomplished template 
+-Photo documentation
+Scanned copy of the ff:
+-Proposal’s Brief of the Program/activity
+-Copy of Activity report
+-Copy of the program
+-Copy of Certificate of participation and or speakership from the beneficiary
+-Copy of attendance sheets per ESCE activity 
+Photo documentation
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accomplished template 
+Scanned copy of MOA/MOU
+Photo documentation
+Other proof of activities conducted 
+Proof of activities delivered via alternative modalities
+Scanned copy of the certification of regular broadcast from the TV or radio station of the said extension activity,
+Electronic copy of print modules and its evidence of distribution
+Evidence of at least 5 recorded broadcasts
+</t>
+  </si>
+  <si>
+    <t>- Impact assessment reports</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-Accomplished template for 
+-Scanned copy of the following:
+-CSC Certification on the PRIME- HRM level of the agency
+-Personnel Development Program
+-Personnel ProfileScanned copy of the following:
+-board-approved Internal selection and promotion guidelines;
+-board-approved personnel sustainability plan;
+-summary of filled up positions
+Scanned copy of the following:
+- HRD Plan
+- Summary of implementation/ accomplishmentsScanned copy of CSC-recognized PRAISE
+Scanned copy of AO 25 Report/certification or PREXC
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-Accomplished template
+-Scanned copy of the following:
+- duly received board-approved LUDIP by CHED Regional Office
+- duly received draft LUDIP by CHED Central Office
+-Scanned copy of the following:
+- transmittal letter duly received Report of Physical Count of PPE (RPCPPE) submitted to COA per year
+- AAR
+-Scanned copy of the following:
+- special order or its equivalent on the designation of a disposal committee.
+- Latest proof of disposal of non- serviceable PPEs report
+- AAR
+-Scanned copy of the following:
+- transmittal letter duly received Report of Physical Count of PPE (RPCPPE) submitted to COA per year
+- AAR
+- Policy on supplies and materials management
+- Proof of Supplies and Materials management system
+- Sample of report generated from the supplies and materials management system
+- Supplies and inventory report submitted to COA
+-Scanned copy of the following:
+- Board-approved Records and Archives Management duly approved by the NAP
+- Archive Certification
+- AAR
+-Scanned copy of the following:
+- Board approved Financial Operations Manual
+- Board approved PRE or WFP or equivalent
+- APP
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-Accomplished template for Scanned copy of the following:
+- Financial Accountability Report (FAR) No. 1, 1A, 1B
+- procurement monitoring report and APP
+-Scanned copy of the following:
+- FAR 2, 2A, 5, 6
+- Report (GPPB)
+- board-approved budget proposal/s
+-Scanned copy of the following:
+- aging schedule report entitled “Due to National Govt Agencies (NGAs)/non-govt org (NGOs)” as submitted to COA
+- Agency Submitted Summary Report of Expenses
+- Liquidation Report following the prescribed COA template
+- MOAD
+-Accomplished template
+-Scanned copy of Annual Audit Report per year of the period covered
+</t>
+  </si>
+  <si>
+    <t>-Accomplished template</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accomplished template 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-Accomplished template 
+</t>
   </si>
 </sst>
 </file>
@@ -573,8 +806,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -855,10 +1089,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E94"/>
+  <dimension ref="A1:H94"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="8" max="8" width="35" style="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -874,8 +1111,11 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H1" s="1" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -891,32 +1131,44 @@
       <c r="E2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H2" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H3" s="1" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C4">
         <v>1.2</v>
       </c>
       <c r="E4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H4" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C5">
         <v>1.3</v>
       </c>
       <c r="E5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H5" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
         <v>12</v>
       </c>
@@ -926,16 +1178,22 @@
       <c r="E6" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H6" s="1" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
         <v>14</v>
       </c>
       <c r="E7" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H7" s="1" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C8">
         <v>1.4</v>
       </c>
@@ -946,7 +1204,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C9">
         <v>1.5</v>
       </c>
@@ -954,7 +1212,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
         <v>18</v>
       </c>
@@ -965,7 +1223,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
         <v>20</v>
       </c>
@@ -973,7 +1231,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
         <v>22</v>
       </c>
@@ -981,7 +1239,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
         <v>24</v>
       </c>
@@ -989,7 +1247,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
         <v>26</v>
       </c>
@@ -997,7 +1255,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C15">
         <v>1.6</v>
       </c>
@@ -1008,7 +1266,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>29</v>
       </c>
@@ -1024,8 +1282,11 @@
       <c r="E16" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="17" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="H16" s="1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="17" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C17">
         <v>2.2000000000000002</v>
       </c>
@@ -1035,24 +1296,33 @@
       <c r="E17" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="18" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="H17" s="1" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="18" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C18" t="s">
         <v>32</v>
       </c>
       <c r="E18" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="19" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="H18" s="1" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="19" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C19" t="s">
         <v>34</v>
       </c>
       <c r="E19" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="20" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="H19" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="20" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C20">
         <v>2.2999999999999998</v>
       </c>
@@ -1060,7 +1330,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C21" t="s">
         <v>37</v>
       </c>
@@ -1070,24 +1340,33 @@
       <c r="E21" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="22" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="H21" s="1" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="22" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C22" t="s">
         <v>39</v>
       </c>
       <c r="E22" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="23" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="H22" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="23" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C23" t="s">
         <v>41</v>
       </c>
       <c r="E23" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="24" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="H23" s="1" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="24" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C24">
         <v>2.4</v>
       </c>
@@ -1097,8 +1376,11 @@
       <c r="E24" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="25" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="H24" s="1" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="25" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C25">
         <v>2.5</v>
       </c>
@@ -1109,7 +1391,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="26" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C26" t="s">
         <v>45</v>
       </c>
@@ -1117,7 +1399,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="27" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C27" t="s">
         <v>47</v>
       </c>
@@ -1125,7 +1407,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="28" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C28">
         <v>2.6</v>
       </c>
@@ -1136,7 +1418,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="29" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C29" t="s">
         <v>50</v>
       </c>
@@ -1144,7 +1426,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="30" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C30">
         <v>2.7</v>
       </c>
@@ -1155,7 +1437,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="31" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C31">
         <v>2.8</v>
       </c>
@@ -1166,7 +1448,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="32" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C32" t="s">
         <v>54</v>
       </c>
@@ -1174,7 +1456,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C33" t="s">
         <v>56</v>
       </c>
@@ -1182,7 +1464,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C34" t="s">
         <v>58</v>
       </c>
@@ -1190,7 +1472,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C35" t="s">
         <v>60</v>
       </c>
@@ -1198,7 +1480,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C36" t="s">
         <v>62</v>
       </c>
@@ -1206,7 +1488,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C37" t="s">
         <v>64</v>
       </c>
@@ -1214,7 +1496,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C38" t="s">
         <v>66</v>
       </c>
@@ -1222,7 +1504,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>68</v>
       </c>
@@ -1238,24 +1520,33 @@
       <c r="E39" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H39" s="1" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C40" t="s">
         <v>70</v>
       </c>
       <c r="E40" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H40" s="1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C41" t="s">
         <v>72</v>
       </c>
       <c r="E41" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H41" s="1" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C42" t="s">
         <v>74</v>
       </c>
@@ -1263,7 +1554,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C43" t="s">
         <v>76</v>
       </c>
@@ -1271,7 +1562,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C44" t="s">
         <v>78</v>
       </c>
@@ -1279,7 +1570,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C45">
         <v>3.2</v>
       </c>
@@ -1290,7 +1581,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C46" t="s">
         <v>81</v>
       </c>
@@ -1298,7 +1589,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C47" t="s">
         <v>83</v>
       </c>
@@ -1306,7 +1597,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C48" t="s">
         <v>85</v>
       </c>
@@ -1314,7 +1605,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C49">
         <v>3.3</v>
       </c>
@@ -1325,7 +1616,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C50" t="s">
         <v>88</v>
       </c>
@@ -1333,7 +1624,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C51" t="s">
         <v>90</v>
       </c>
@@ -1341,7 +1632,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C52" t="s">
         <v>92</v>
       </c>
@@ -1349,7 +1640,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C53" t="s">
         <v>94</v>
       </c>
@@ -1357,7 +1648,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C54" t="s">
         <v>96</v>
       </c>
@@ -1365,7 +1656,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>98</v>
       </c>
@@ -1381,8 +1672,11 @@
       <c r="E55" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H55" s="1" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C56" t="s">
         <v>100</v>
       </c>
@@ -1390,31 +1684,40 @@
         <v>101</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C57" t="s">
         <v>102</v>
       </c>
       <c r="E57" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H57" s="1" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C58" t="s">
         <v>104</v>
       </c>
       <c r="E58" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H58" s="1" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C59">
         <v>4.2</v>
       </c>
       <c r="E59" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H59" s="1" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C60" t="s">
         <v>107</v>
       </c>
@@ -1422,7 +1725,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C61" t="s">
         <v>109</v>
       </c>
@@ -1430,7 +1733,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C62" t="s">
         <v>111</v>
       </c>
@@ -1438,7 +1741,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C63" t="s">
         <v>113</v>
       </c>
@@ -1446,7 +1749,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C64">
         <v>4.4000000000000004</v>
       </c>
@@ -1454,7 +1757,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C65" t="s">
         <v>116</v>
       </c>
@@ -1462,7 +1765,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C66" t="s">
         <v>118</v>
       </c>
@@ -1470,7 +1773,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C67" t="s">
         <v>120</v>
       </c>
@@ -1478,7 +1781,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C68" t="s">
         <v>122</v>
       </c>
@@ -1486,7 +1789,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>124</v>
       </c>
@@ -1502,8 +1805,11 @@
       <c r="E69" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H69" s="1" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C70">
         <v>5.2</v>
       </c>
@@ -1513,8 +1819,11 @@
       <c r="E70" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H70" s="1" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C71" t="s">
         <v>127</v>
       </c>
@@ -1522,7 +1831,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C72" t="s">
         <v>129</v>
       </c>
@@ -1530,7 +1839,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C73" t="s">
         <v>131</v>
       </c>
@@ -1538,7 +1847,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C74" t="s">
         <v>133</v>
       </c>
@@ -1546,7 +1855,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C75" t="s">
         <v>135</v>
       </c>
@@ -1554,7 +1863,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C76" t="s">
         <v>137</v>
       </c>
@@ -1562,7 +1871,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C77" t="s">
         <v>139</v>
       </c>
@@ -1570,7 +1879,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C78">
         <v>5.3</v>
       </c>
@@ -1580,8 +1889,11 @@
       <c r="E78" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H78" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C79" t="s">
         <v>142</v>
       </c>
@@ -1589,7 +1901,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C80" t="s">
         <v>144</v>
       </c>
@@ -1597,7 +1909,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="81" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C81" t="s">
         <v>146</v>
       </c>
@@ -1605,7 +1917,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="82" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C82" t="s">
         <v>148</v>
       </c>
@@ -1613,7 +1925,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="83" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C83" t="s">
         <v>150</v>
       </c>
@@ -1621,7 +1933,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="84" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C84" t="s">
         <v>152</v>
       </c>
@@ -1629,7 +1941,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="85" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C85" t="s">
         <v>154</v>
       </c>
@@ -1637,7 +1949,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="86" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C86" t="s">
         <v>156</v>
       </c>
@@ -1645,7 +1957,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="87" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C87">
         <v>5.4</v>
       </c>
@@ -1655,8 +1967,11 @@
       <c r="E87" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="88" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="H87" s="1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="88" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C88">
         <v>5.5</v>
       </c>
@@ -1666,16 +1981,22 @@
       <c r="E88" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="89" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="H88" s="1" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="89" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C89" t="s">
         <v>160</v>
       </c>
       <c r="E89" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="90" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="H89" s="1" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="90" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C90" t="s">
         <v>162</v>
       </c>
@@ -1683,7 +2004,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="91" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C91">
         <v>5.6</v>
       </c>
@@ -1691,7 +2012,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="92" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C92" t="s">
         <v>165</v>
       </c>
@@ -1699,7 +2020,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="93" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C93" t="s">
         <v>167</v>
       </c>
@@ -1707,7 +2028,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="94" spans="3:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C94" t="s">
         <v>169</v>
       </c>

</xml_diff>